<commit_message>
Add the mPBalk scenario macro to the ProModel tables
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018RXhixPdKWR4gEynjbfZmu
</commit_message>
<xml_diff>
--- a/codespace/promodel_inputs/ProModel_tables.xlsx
+++ b/codespace/promodel_inputs/ProModel_tables.xlsx
@@ -4116,14 +4116,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="47" customWidth="1" min="5" max="5"/>
+    <col width="49" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -4252,58 +4252,88 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>mSiteLimitkW</t>
+          <t>mPBalk</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>150</v>
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>20 - 150</t>
+          <t>0.5 - 1.0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>probability</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>site power cap (stage 5)</t>
+          <t>leave at once when all EVSEs are busy (stage 5)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Lee et al. 2021a; acnportal (150 kVA transformer)</t>
+          <t>assumption (R02)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>mSiteLimitkW</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>150</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>20 - 150</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>site power cap (stage 5)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Lee et al. 2021a; acnportal (150 kVA transformer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>mPolicy</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B7" t="n">
         <v>1</v>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>1 uncontrolled / 2 equal share / 3 earliest departure first / 4 move after charge</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>charging policy (stage 5)</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>proposal</t>
         </is>

</xml_diff>

<commit_message>
Draw the user class after dwell to keep the dwell-energy correlation
Unclaimed sessions are mostly short stays (median dwell 2.6 h against
5.8 h for claimed ones): 27.1% of 0-2 h stays are unclaimed but only
7.0% of 10-24 h stays. Drawing the class independently of dwell put
low-energy unclaimed sessions on long stays and weakened the dwell-energy
correlation of the model (Spearman 0.22 over all sessions, observed
0.37). Drawing it after dwell from the share per dwell bin raises it to
0.31 and keeps the overall unclaimed share (15.3%, observed 15.4%).

- fit_acn.py: writes unclaimed_share_by_dwell (same bins as the energy
  fits). No other result changes.
- export_promodel_tables.py: new sheet "Unclaimed by dwell".
- make_md.py: the aUserClass row gives the shares by dwell bin.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018RXhixPdKWR4gEynjbfZmu
</commit_message>
<xml_diff>
--- a/codespace/promodel_inputs/ProModel_tables.xlsx
+++ b/codespace/promodel_inputs/ProModel_tables.xlsx
@@ -15,8 +15,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Energy" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Empirical tables" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User class" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Macros" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Announced inputs" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unclaimed by dwell" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Macros" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Announced inputs" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -521,35 +522,46 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>User distribution dUserClass (discrete)</t>
+          <t>User distribution dUserClass (discrete): overall shares, for reference and stage 4</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Macros</t>
+          <t>Unclaimed by dwell</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Scenario macros with baseline and test values</t>
+          <t>Share of unclaimed sessions by dwell bin: aUserClass is drawn after aDwell from these</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Macros</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Scenario macros with baseline and test values</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Announced inputs</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Announced-input error quantiles (for aDepAnnounced and aEnergyReq in later stages)</t>
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -725,6 +737,240 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="49" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Macro</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Scenario values</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Used in</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>mPorts</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>54</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>30 / 42 / 54 / 66</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>EVSEs</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>EVSE_BANK capacity</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Garage 01 has 54 Level-2 EVSEs; proposal factor levels</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>mRate</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>3.17 / 4.8 / 6.66</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>constant effective charging rate (stages 1-3)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>median observed kWh per charging hour (n=16140); 4.8 = vehicle-rate mix mean; 6.66 = EVSE rating</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>mDemand</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0.8 / 1.0 / 1.2 / 1.5</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>x daily arrivals</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Arrivals Qty Each</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>proposal (R17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mPBalk</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0.5 - 1.0</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>probability</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>leave at once when all EVSEs are busy (stage 5)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>assumption (R02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>mSiteLimitkW</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>150</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>20 - 150</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>site power cap (stage 5)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Lee et al. 2021a; acnportal (150 kVA transformer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>mPolicy</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1 uncontrolled / 2 equal share / 3 earliest departure first / 4 move after charge</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>charging policy (stage 5)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>proposal</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4116,227 +4362,83 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="49" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Macro</t>
+          <t>Dwell (h)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Baseline</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Scenario values</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Used in</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Source</t>
+          <t>Unclaimed share %</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>mPorts</t>
+          <t>0-2</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>54</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>30 / 42 / 54 / 66</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>EVSEs</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>EVSE_BANK capacity</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Garage 01 has 54 Level-2 EVSEs; proposal factor levels</t>
-        </is>
+        <v>27.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>mRate</t>
+          <t>2-4</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3.17</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>3.17 / 4.8 / 6.66</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>kW</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>constant effective charging rate (stages 1-3)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>median observed kWh per charging hour (n=16140); 4.8 = vehicle-rate mix mean; 6.66 = EVSE rating</t>
-        </is>
+        <v>18.2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>mDemand</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>0.8 / 1.0 / 1.2 / 1.5</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>x daily arrivals</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Arrivals Qty Each</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>proposal (R17)</t>
-        </is>
+        <v>13.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>mPBalk</t>
+          <t>6-8</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>0.5 - 1.0</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>probability</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>leave at once when all EVSEs are busy (stage 5)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>assumption (R02)</t>
-        </is>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>mSiteLimitkW</t>
+          <t>8-10</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>150</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>20 - 150</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>kW</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>site power cap (stage 5)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Lee et al. 2021a; acnportal (150 kVA transformer)</t>
-        </is>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>mPolicy</t>
+          <t>10-24</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1 uncontrolled / 2 equal share / 3 earliest departure first / 4 move after charge</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>charging policy (stage 5)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>proposal</t>
-        </is>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add P95 and P99 to the empirical tables and cap energy need at 6.66 kW x dwell
With deciles alone, linear interpolation over the top 10% runs to the
maximum and inflates the table means (+6-8% for the morning dwell groups,
+38% for unclaimed kWh). The empirical user distributions now use
P0-P90 by 10, P95, P99 and P100, which brings the gap to 0.2-3.6%.
acn_fits.json stores these as table_points instead of deciles_0_to_100;
no other value changes.

The draft also states that energy need is capped at 6.66 kW x dwell
after it is drawn: energy is drawn independently of dwell inside a dwell
bin, so about 6.6% of draws could not be delivered even at the port
rating, which never happens in the data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018RXhixPdKWR4gEynjbfZmu
</commit_message>
<xml_diff>
--- a/codespace/promodel_inputs/ProModel_tables.xlsx
+++ b/codespace/promodel_inputs/ProModel_tables.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Continuous cumulative user distributions for the groups whose best fit has KS &gt; 0.1</t>
+          <t>Continuous cumulative user distributions for the groups whose best fit has KS &gt; 0.1 (P0-P90 by 10, P95, P99, P100)</t>
         </is>
       </c>
     </row>
@@ -3453,7 +3453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -3676,46 +3676,46 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D12" t="n">
-        <v>22.47</v>
+        <v>13.63</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>dDwellWD0709</t>
+          <t>dDwellWD0007</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>weekday 07-09</t>
+          <t>weekday 00-07</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="D13" t="n">
-        <v>0.11</v>
+        <v>18.23</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dDwellWD0709</t>
+          <t>dDwellWD0007</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>weekday 07-09</t>
+          <t>weekday 00-07</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="D14" t="n">
-        <v>2.79</v>
+        <v>22.47</v>
       </c>
     </row>
     <row r="15">
@@ -3730,10 +3730,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>4.21</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="16">
@@ -3748,10 +3748,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="D16" t="n">
-        <v>6.13</v>
+        <v>2.79</v>
       </c>
     </row>
     <row r="17">
@@ -3766,10 +3766,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D17" t="n">
-        <v>7.67</v>
+        <v>4.21</v>
       </c>
     </row>
     <row r="18">
@@ -3784,10 +3784,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="D18" t="n">
-        <v>8.42</v>
+        <v>6.13</v>
       </c>
     </row>
     <row r="19">
@@ -3802,10 +3802,10 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="D19" t="n">
-        <v>8.789999999999999</v>
+        <v>7.67</v>
       </c>
     </row>
     <row r="20">
@@ -3820,10 +3820,10 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="D20" t="n">
-        <v>9.109999999999999</v>
+        <v>8.42</v>
       </c>
     </row>
     <row r="21">
@@ -3838,10 +3838,10 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="D21" t="n">
-        <v>9.59</v>
+        <v>8.789999999999999</v>
       </c>
     </row>
     <row r="22">
@@ -3856,10 +3856,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="D22" t="n">
-        <v>10.27</v>
+        <v>9.109999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -3874,82 +3874,82 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="D23" t="n">
-        <v>22.32</v>
+        <v>9.59</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>dDwellWD0911</t>
+          <t>dDwellWD0709</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>weekday 09-11</t>
+          <t>weekday 07-09</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="D24" t="n">
-        <v>0.09</v>
+        <v>10.27</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>dDwellWD0911</t>
+          <t>dDwellWD0709</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>weekday 09-11</t>
+          <t>weekday 07-09</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>10</v>
+        <v>95</v>
       </c>
       <c r="D25" t="n">
-        <v>1.98</v>
+        <v>11.06</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>dDwellWD0911</t>
+          <t>dDwellWD0709</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>weekday 09-11</t>
+          <t>weekday 07-09</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="D26" t="n">
-        <v>3.9</v>
+        <v>12.86</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>dDwellWD0911</t>
+          <t>dDwellWD0709</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>weekday 09-11</t>
+          <t>weekday 07-09</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="D27" t="n">
-        <v>6.11</v>
+        <v>22.32</v>
       </c>
     </row>
     <row r="28">
@@ -3964,10 +3964,10 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>6.98</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="29">
@@ -3982,10 +3982,10 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="D29" t="n">
-        <v>7.5</v>
+        <v>1.98</v>
       </c>
     </row>
     <row r="30">
@@ -4000,10 +4000,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="D30" t="n">
-        <v>7.95</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="31">
@@ -4018,10 +4018,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="D31" t="n">
-        <v>8.43</v>
+        <v>6.11</v>
       </c>
     </row>
     <row r="32">
@@ -4036,10 +4036,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="D32" t="n">
-        <v>8.960000000000001</v>
+        <v>6.98</v>
       </c>
     </row>
     <row r="33">
@@ -4054,10 +4054,10 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="D33" t="n">
-        <v>9.699999999999999</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="34">
@@ -4072,118 +4072,118 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="D34" t="n">
-        <v>23.92</v>
+        <v>7.95</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>dEnergyUnclaimed</t>
+          <t>dDwellWD0911</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>unclaimed (30-min auto stop)</t>
+          <t>weekday 09-11</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="D35" t="n">
-        <v>0.5</v>
+        <v>8.43</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>dEnergyUnclaimed</t>
+          <t>dDwellWD0911</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>unclaimed (30-min auto stop)</t>
+          <t>weekday 09-11</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="D36" t="n">
-        <v>0.77</v>
+        <v>8.960000000000001</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>dEnergyUnclaimed</t>
+          <t>dDwellWD0911</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>unclaimed (30-min auto stop)</t>
+          <t>weekday 09-11</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="D37" t="n">
-        <v>0.83</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>dEnergyUnclaimed</t>
+          <t>dDwellWD0911</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>unclaimed (30-min auto stop)</t>
+          <t>weekday 09-11</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>30</v>
+        <v>95</v>
       </c>
       <c r="D38" t="n">
-        <v>0.85</v>
+        <v>10.47</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>dEnergyUnclaimed</t>
+          <t>dDwellWD0911</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>unclaimed (30-min auto stop)</t>
+          <t>weekday 09-11</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>40</v>
+        <v>99</v>
       </c>
       <c r="D39" t="n">
-        <v>0.87</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>dEnergyUnclaimed</t>
+          <t>dDwellWD0911</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>unclaimed (30-min auto stop)</t>
+          <t>weekday 09-11</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D40" t="n">
-        <v>0.89</v>
+        <v>23.92</v>
       </c>
     </row>
     <row r="41">
@@ -4198,10 +4198,10 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="D41" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="42">
@@ -4216,10 +4216,10 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="D42" t="n">
-        <v>0.93</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="43">
@@ -4234,10 +4234,10 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="D43" t="n">
-        <v>0.97</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="44">
@@ -4252,10 +4252,10 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="D44" t="n">
-        <v>1.19</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="45">
@@ -4270,9 +4270,153 @@
         </is>
       </c>
       <c r="C45" t="n">
+        <v>40</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>dEnergyUnclaimed</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>unclaimed (30-min auto stop)</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>50</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>dEnergyUnclaimed</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>unclaimed (30-min auto stop)</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>60</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>dEnergyUnclaimed</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>unclaimed (30-min auto stop)</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>70</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>dEnergyUnclaimed</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>unclaimed (30-min auto stop)</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>80</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0.97</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>dEnergyUnclaimed</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>unclaimed (30-min auto stop)</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>90</v>
+      </c>
+      <c r="D50" t="n">
+        <v>1.19</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>dEnergyUnclaimed</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>unclaimed (30-min auto stop)</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>95</v>
+      </c>
+      <c r="D51" t="n">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>dEnergyUnclaimed</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>unclaimed (30-min auto stop)</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>99</v>
+      </c>
+      <c r="D52" t="n">
+        <v>4.92</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>dEnergyUnclaimed</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>unclaimed (30-min auto stop)</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
         <v>100</v>
       </c>
-      <c r="D45" t="n">
+      <c r="D53" t="n">
         <v>11.81</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Describe the per-car charging rate for stages 1-3
A constant rate either leaves about 23% of cars short at 3.17 kW or
halves the charging time at 6.66 kW. Each car now charges at mRate
(3.17 kW, the observed median) unless it needs more to finish before it
leaves: at service start the rate is aEnergyNeed / remaining time,
between mRate and 6.66 kW. With no queue every car is full, delivered
energy is 97.5% of the data, and claimed sessions charge 2.6 h on
average (2.7 h observed). The draft section 3.5 and the mRate row of
the Macros sheet say so.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018RXhixPdKWR4gEynjbfZmu
</commit_message>
<xml_diff>
--- a/codespace/promodel_inputs/ProModel_tables.xlsx
+++ b/codespace/promodel_inputs/ProModel_tables.xlsx
@@ -749,7 +749,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="49" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -836,7 +836,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>constant effective charging rate (stages 1-3)</t>
+          <t>normal charging rate; at service start code B raises a car's rate to aEnergyNeed / remaining time when needed, up to 6.66 kW</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">

</xml_diff>